<commit_message>
Improve review and tolerance workbook readability without changing test content
</commit_message>
<xml_diff>
--- a/UnitTest/VCU_VcScHv_SWUT.xlsx
+++ b/UnitTest/VCU_VcScHv_SWUT.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TCSD" sheetId="1" r:id="R1bed50af6b0949be"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tolerance" sheetId="2" r:id="R161f3a9f08824be5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TCSD" sheetId="1" r:id="R6ae040d30c1142ee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tolerance" sheetId="2" r:id="Ra60406adf78a4459"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -11521,14 +11521,14 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="18" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="18" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="18" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="18" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="18" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="54" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="28" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="28" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="28" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="28" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" ht="42" customHeight="1">
+    <x:row r="1" ht="62" customHeight="1">
       <x:c r="A1" s="4" t="str">
         <x:v>Output Interface</x:v>
       </x:c>

</xml_diff>